<commit_message>
Clarify TraceGuide study group labels
</commit_message>
<xml_diff>
--- a/docs/TraceGuide_Block_Survey_Data_Workbook.xlsx
+++ b/docs/TraceGuide_Block_Survey_Data_Workbook.xlsx
@@ -543,27 +543,27 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Group</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Order</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>First block</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Second block</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Participant codes</t>
         </is>
@@ -572,7 +572,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>G1</t>
+          <t>Group 1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -582,12 +582,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>A: S1-T1, S1-T2</t>
+          <t>Baseline: S1-T1, S1-T2</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>B: S2-T1, S2-T2</t>
+          <t>TraceGuide: S2-T1, S2-T2</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -599,7 +599,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>G2</t>
+          <t>Group 2</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -609,12 +609,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>B: S1-T1, S1-T2</t>
+          <t>TraceGuide: S1-T1, S1-T2</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>A: S2-T1, S2-T2</t>
+          <t>Baseline: S2-T1, S2-T2</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">

</xml_diff>